<commit_message>
v1.2: Figure S1 script, curated names, Dataset wording and integrity check
</commit_message>
<xml_diff>
--- a/curation/S5_curated_regulators.xlsx
+++ b/curation/S5_curated_regulators.xlsx
@@ -426,7 +426,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -434,7 +433,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -490,7 +488,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -546,7 +543,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -2820,7 +2816,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>dnaA</t>
+          <t>DnaA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3068,7 +3064,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>sigC</t>
+          <t>SigA5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3326,7 +3322,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>nusA</t>
+          <t>NusA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3503,7 +3499,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>nrdR</t>
+          <t>NrdR</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3943,7 +3939,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>pyrR</t>
+          <t>PyrR</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4002,7 +3998,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>sfsA</t>
+          <t>SfsA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4066,7 +4062,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>sufR</t>
+          <t>SufR</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4152,7 +4148,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>lexA</t>
+          <t>LexA</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4393,7 +4389,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>hrcA</t>
+          <t>HrcA</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5208,7 +5204,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>nusG</t>
+          <t>NusG</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5390,7 +5386,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>rpoD</t>
+          <t>SigA1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5422,7 +5418,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>lexA</t>
+          <t>LexA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5572,7 +5568,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>hrcA</t>
+          <t>HrcA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5744,7 +5740,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>sigC</t>
+          <t>SigA5</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5808,7 +5804,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>pyrR</t>
+          <t>PyrR</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -5899,7 +5895,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>nrdR</t>
+          <t>NrdR</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -5931,7 +5927,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>nusA</t>
+          <t>NusA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6275,7 +6271,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>sfsA</t>
+          <t>SfsA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -6862,7 +6858,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>sufR</t>
+          <t>SufR</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -6975,7 +6971,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>kaiC</t>
+          <t>KaiC2</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -7007,7 +7003,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>nusB</t>
+          <t>NusB</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -7120,7 +7116,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>dnaA</t>
+          <t>DnaA</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">

</xml_diff>